<commit_message>
Exercise 2.A normalization complete
</commit_message>
<xml_diff>
--- a/week-02/Ex2A_events_normalized.xlsx
+++ b/week-02/Ex2A_events_normalized.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ricar\Documents\DataAnalytics\week-02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152C6487-406D-4385-97FC-5A005B6C999F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D186E44D-F21F-4201-AC06-CCD42BB8309A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="131">
   <si>
     <t>Event ID</t>
   </si>
@@ -417,6 +417,17 @@
   </si>
   <si>
     <t>Venues</t>
+  </si>
+  <si>
+    <t>Managers</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>**AI Feedback Reflection**
+The AI review confirmed that my four tables were correctly normalized, with unique primary keys and consistent relationships between them. One helpful suggestion was to remove unnecessary spaces from text fields to improve data consistency. It also recommended treating ZIP codes as text to preserve leading zeros.
+I did not need to change my table structure because the review found no duplicate primary keys, missing records, or broken relationships. The ZIP code recommendation is useful for future datasets, but it does not affect the existing values in this spreadsheet.</t>
   </si>
 </sst>
 </file>
@@ -921,13 +932,16 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1303,12 +1317,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FA38BEC-78EC-44DC-83F3-AA711D021920}">
-  <dimension ref="A1:Q67"/>
+  <dimension ref="A1:Q78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
     <col min="2" max="2" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
@@ -2509,17 +2523,167 @@
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B50" s="3"/>
+      <c r="B50" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B51" t="s">
+        <v>105</v>
+      </c>
+      <c r="C51" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B52" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B53" t="s">
+        <v>9</v>
+      </c>
+      <c r="C53" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B54" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B55" t="s">
+        <v>20</v>
+      </c>
+      <c r="C55" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B56" t="s">
+        <v>23</v>
+      </c>
+      <c r="C56" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B57" t="s">
+        <v>29</v>
+      </c>
+      <c r="C57" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B67" s="3"/>
+      <c r="B67" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B68" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="5">
+        <v>7</v>
+      </c>
+      <c r="B69" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="5">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="5">
+        <v>3</v>
+      </c>
+      <c r="B71" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="5">
+        <v>6</v>
+      </c>
+      <c r="B72" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="5">
+        <v>4</v>
+      </c>
+      <c r="B73" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="5">
+        <v>5</v>
+      </c>
+      <c r="B74" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="5">
+        <v>1</v>
+      </c>
+      <c r="B75" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A78" s="6" t="s">
+        <v>130</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J19:J29">

</xml_diff>